<commit_message>
ios: screenshot dell'app aggiornati per lo store, didascalia EN 02 neutra
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_store_tradotto.xlsx
+++ b/ios/localizzazione/NEAT_store_tradotto.xlsx
@@ -1402,7 +1402,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>In walking minutes and kilometers</t>
+          <t>In walking minutes and distance</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -1449,7 +1449,11 @@
         <f>"EN: "&amp;LEN(F10)&amp;CHAR(10)&amp;"ES: "&amp;LEN(G10)&amp;CHAR(10)&amp;"FR: "&amp;LEN(H10)&amp;CHAR(10)&amp;"DE: "&amp;LEN(I10)&amp;CHAR(10)&amp;"PT-BR: "&amp;LEN(J10)&amp;CHAR(10)&amp;"JA: "&amp;LEN(K10)&amp;CHAR(10)&amp;"KO: "&amp;LEN(L10)&amp;CHAR(10)&amp;"ZH-Hans: "&amp;LEN(M10)&amp;CHAR(10)&amp;"ZH-Hant: "&amp;LEN(N10)</f>
         <v/>
       </c>
-      <c r="P10" s="6" t="n"/>
+      <c r="P10" s="6" t="inlineStr">
+        <is>
+          <t>COORDINAMENTO: EN neutra (miglia negli USA/UK, km altrove).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">

</xml_diff>

<commit_message>
ios 1.1: screenshot 6 e pagina Salute dell'introduzione con la nuova promessa
«I TUOI DATI SONO SOLO TUOI / Nessuno li vede, nemmeno noi» nel foglio dello store; nell'introduzione «I tuoi dati
non lasciano mai il tuo account» (traduzioni bozza, cataloghi rigenerati). Prompt per ChatGPT esteso, prompt per
Claude Design dello screenshot 6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_store_tradotto.xlsx
+++ b/ios/localizzazione/NEAT_store_tradotto.xlsx
@@ -1956,7 +1956,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>I TUOI DATI RESTANO SUL TUO IPHONE</t>
+          <t>I TUOI DATI SONO SOLO TUOI</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Nessun dato lascia il telefono</t>
+          <t>Nessuno li vede, nemmeno noi</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">

</xml_diff>